<commit_message>
update birthdate card (#442) 1dc930f91b94c26cde184a75bf4a709c271ea861
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-tddui-patient.xlsx
+++ b/main/ig/StructureDefinition-tddui-patient.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-26T16:06:51+00:00</t>
+    <t>2026-02-27T10:48:32+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -24458,7 +24458,7 @@
       </c>
       <c r="E174" s="2"/>
       <c r="F174" t="s" s="2">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="G174" t="s" s="2">
         <v>91</v>

</xml_diff>